<commit_message>
Clean dummy survey entries, filter Dausa working sample (N=50), and generate 4 client Excel files
</commit_message>
<xml_diff>
--- a/Projects/CmF_SHG_Women_Entrepreneurs/reports/district_analysis/All_Rajasthan/excel/All_Rajasthan_Survey_Analysis_Master.xlsx
+++ b/Projects/CmF_SHG_Women_Entrepreneurs/reports/district_analysis/All_Rajasthan/excel/All_Rajasthan_Survey_Analysis_Master.xlsx
@@ -816,13 +816,13 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>2563000</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>284777.7777777778</v>
+        <v>183071.4285714286</v>
       </c>
       <c r="G4" s="7" t="n">
         <v>285000</v>
@@ -881,13 +881,13 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E5" s="7" t="n">
         <v>2703000</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>450500</v>
+        <v>245727.2727272727</v>
       </c>
       <c r="G5" s="7" t="n">
         <v>520000</v>
@@ -946,13 +946,13 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>483000</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>241500</v>
+        <v>80500</v>
       </c>
       <c r="G6" s="7" t="n">
         <v>92000</v>
@@ -1490,16 +1490,16 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>3880501</v>
+        <v>3862501</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>228264.7647058823</v>
+        <v>203289.5263157895</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>1541501</v>
+        <v>1523501</v>
       </c>
       <c r="H14" s="7" t="n">
         <v>258000</v>
@@ -1555,13 +1555,13 @@
         </is>
       </c>
       <c r="D15" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E15" s="7" t="n">
         <v>392100</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>130700</v>
+        <v>98025</v>
       </c>
       <c r="G15" s="7" t="n">
         <v>15000</v>
@@ -1814,8 +1814,8 @@
           <t>Tent house</t>
         </is>
       </c>
-      <c r="D19" s="9" t="n">
-        <v>0</v>
+      <c r="D19" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="E19" s="8" t="n">
         <v>0</v>
@@ -2229,13 +2229,13 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E25" s="7" t="n">
         <v>62300</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>62300</v>
+        <v>31150</v>
       </c>
       <c r="G25" s="7" t="n">
         <v>17000</v>
@@ -2424,13 +2424,13 @@
         </is>
       </c>
       <c r="D28" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E28" s="7" t="n">
         <v>1033601</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>258400.25</v>
+        <v>206720.2</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>270000</v>
@@ -3883,19 +3883,19 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="G5" s="6" t="n">
-        <v>2</v>
-      </c>
       <c r="H5" s="6" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6">
@@ -3909,7 +3909,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>1</v>
@@ -3918,10 +3918,10 @@
         <v>1</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
@@ -3941,13 +3941,13 @@
         <v>0</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -4156,17 +4156,17 @@
       <c r="D15" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="E15" s="9" t="n">
-        <v>0</v>
+      <c r="E15" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16">
@@ -4186,13 +4186,13 @@
         <v>0</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G16" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
@@ -4292,11 +4292,11 @@
       <c r="F20" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>0</v>
+      <c r="G20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -4450,8 +4450,8 @@
           <t>Dairy shop/Milk collection centre</t>
         </is>
       </c>
-      <c r="D26" s="9" t="n">
-        <v>0</v>
+      <c r="D26" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="E26" s="9" t="n">
         <v>0</v>
@@ -4463,7 +4463,7 @@
         <v>0</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -4535,13 +4535,13 @@
         <v>0</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G29" s="6" t="n">
         <v>1</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30">
@@ -4761,7 +4761,7 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4801,10 +4801,10 @@
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>0.2142857142857143</v>
+        <v>0.2297297297297297</v>
       </c>
     </row>
     <row r="5">
@@ -4814,10 +4814,10 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>0.2678571428571428</v>
+        <v>0.2702702702702703</v>
       </c>
     </row>
     <row r="6">
@@ -4827,10 +4827,10 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>0.2678571428571428</v>
+        <v>0.3108108108108108</v>
       </c>
     </row>
     <row r="7">
@@ -4840,10 +4840,10 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3108108108108108</v>
       </c>
     </row>
     <row r="8">
@@ -4853,10 +4853,10 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>0.375</v>
+        <v>0.3648648648648649</v>
       </c>
     </row>
     <row r="9">
@@ -4905,10 +4905,10 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>0.2142857142857143</v>
+        <v>0.2297297297297297</v>
       </c>
     </row>
     <row r="14">
@@ -4918,10 +4918,10 @@
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>0.3035714285714285</v>
+        <v>0.3108108108108108</v>
       </c>
     </row>
     <row r="15">
@@ -4931,10 +4931,10 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>0.2142857142857143</v>
+        <v>0.2297297297297297</v>
       </c>
     </row>
     <row r="16">
@@ -4956,11 +4956,11 @@
           <t>I want to source material from different places but I need support</t>
         </is>
       </c>
-      <c r="C17" s="9" t="n">
-        <v>0</v>
+      <c r="C17" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>0</v>
+        <v>0.01351351351351351</v>
       </c>
     </row>
     <row r="18">
@@ -4970,10 +4970,10 @@
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>0.1964285714285714</v>
+        <v>0.2027027027027027</v>
       </c>
     </row>
     <row r="19">
@@ -5030,7 +5030,7 @@
         </is>
       </c>
       <c r="C2" s="27" t="n">
-        <v>56</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3"/>
@@ -5063,10 +5063,10 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.6351351351351351</v>
       </c>
     </row>
     <row r="6">
@@ -5076,10 +5076,10 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3648648648648649</v>
       </c>
     </row>
     <row r="7">
@@ -5127,10 +5127,10 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>0.25</v>
+        <v>0.2297297297297297</v>
       </c>
     </row>
     <row r="11">
@@ -5140,10 +5140,10 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>0.75</v>
+        <v>0.7702702702702703</v>
       </c>
     </row>
     <row r="12">
@@ -5191,10 +5191,10 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>0.3035714285714285</v>
+        <v>0.4054054054054054</v>
       </c>
     </row>
     <row r="16">
@@ -5204,10 +5204,10 @@
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D16" s="25" t="n">
-        <v>0.5</v>
+        <v>0.4324324324324325</v>
       </c>
     </row>
     <row r="17">
@@ -5217,10 +5217,10 @@
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>0.25</v>
+        <v>0.2162162162162162</v>
       </c>
     </row>
     <row r="18">
@@ -5268,10 +5268,10 @@
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>0.9464285714285714</v>
+        <v>0.9594594594594594</v>
       </c>
     </row>
     <row r="22">
@@ -5281,10 +5281,10 @@
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="D22" s="25" t="n">
-        <v>0.9821428571428571</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -5294,10 +5294,10 @@
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.6351351351351351</v>
       </c>
     </row>
     <row r="24">
@@ -5307,10 +5307,10 @@
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D24" s="25" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.05405405405405406</v>
       </c>
     </row>
     <row r="25">
@@ -5323,7 +5323,7 @@
         <v>3</v>
       </c>
       <c r="D25" s="25" t="n">
-        <v>0.05357142857142857</v>
+        <v>0.04054054054054054</v>
       </c>
     </row>
     <row r="26">
@@ -5333,10 +5333,10 @@
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="D26" s="25" t="n">
-        <v>0.9285714285714286</v>
+        <v>0.9459459459459459</v>
       </c>
     </row>
     <row r="27">
@@ -5346,10 +5346,10 @@
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.5405405405405406</v>
       </c>
     </row>
     <row r="28">
@@ -5400,7 +5400,7 @@
         <v>2</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.02702702702702703</v>
       </c>
     </row>
     <row r="32">
@@ -5410,10 +5410,10 @@
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="D32" s="25" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.4189189189189189</v>
       </c>
     </row>
     <row r="33">
@@ -5423,10 +5423,10 @@
         </is>
       </c>
       <c r="C33" s="6" t="n">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="D33" s="25" t="n">
-        <v>0.375</v>
+        <v>0.3783783783783784</v>
       </c>
     </row>
     <row r="34">
@@ -5436,10 +5436,10 @@
         </is>
       </c>
       <c r="C34" s="6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D34" s="25" t="n">
-        <v>0.1071428571428571</v>
+        <v>0.1351351351351351</v>
       </c>
     </row>
     <row r="35">
@@ -5449,10 +5449,10 @@
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D35" s="25" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.04054054054054054</v>
       </c>
     </row>
     <row r="36">
@@ -5513,10 +5513,10 @@
         </is>
       </c>
       <c r="C40" s="6" t="n">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="D40" s="25" t="n">
-        <v>0.9107142857142857</v>
+        <v>0.9459459459459459</v>
       </c>
     </row>
     <row r="41">
@@ -5526,10 +5526,10 @@
         </is>
       </c>
       <c r="C41" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D41" s="25" t="n">
-        <v>0.05357142857142857</v>
+        <v>0.05405405405405406</v>
       </c>
     </row>
     <row r="42">
@@ -5603,10 +5603,10 @@
         </is>
       </c>
       <c r="C47" s="6" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="D47" s="25" t="n">
-        <v>0.3214285714285715</v>
+        <v>0.3378378378378378</v>
       </c>
     </row>
     <row r="48">
@@ -5616,10 +5616,10 @@
         </is>
       </c>
       <c r="C48" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D48" s="25" t="n">
-        <v>0.05357142857142857</v>
+        <v>0.05405405405405406</v>
       </c>
     </row>
     <row r="49">
@@ -5629,10 +5629,10 @@
         </is>
       </c>
       <c r="C49" s="6" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D49" s="25" t="n">
-        <v>0.3928571428571428</v>
+        <v>0.3783783783783784</v>
       </c>
     </row>
     <row r="50">
@@ -5642,10 +5642,10 @@
         </is>
       </c>
       <c r="C50" s="6" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D50" s="25" t="n">
-        <v>0.1964285714285714</v>
+        <v>0.2297297297297297</v>
       </c>
     </row>
     <row r="51">
@@ -5693,10 +5693,10 @@
         </is>
       </c>
       <c r="C54" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D54" s="25" t="n">
-        <v>0.1071428571428571</v>
+        <v>0.1216216216216216</v>
       </c>
     </row>
     <row r="55">
@@ -5709,7 +5709,7 @@
         <v>1</v>
       </c>
       <c r="D55" s="25" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.01351351351351351</v>
       </c>
     </row>
     <row r="56">
@@ -5719,10 +5719,10 @@
         </is>
       </c>
       <c r="C56" s="6" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D56" s="25" t="n">
-        <v>0.25</v>
+        <v>0.2432432432432433</v>
       </c>
     </row>
     <row r="57">
@@ -5732,10 +5732,10 @@
         </is>
       </c>
       <c r="C57" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D57" s="25" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.1486486486486487</v>
       </c>
     </row>
     <row r="58">
@@ -5745,10 +5745,10 @@
         </is>
       </c>
       <c r="C58" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D58" s="25" t="n">
-        <v>0.2142857142857143</v>
+        <v>0.1891891891891892</v>
       </c>
     </row>
     <row r="59">
@@ -5758,10 +5758,10 @@
         </is>
       </c>
       <c r="C59" s="6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D59" s="25" t="n">
-        <v>0.1607142857142857</v>
+        <v>0.1486486486486487</v>
       </c>
     </row>
     <row r="60">
@@ -5784,10 +5784,10 @@
         </is>
       </c>
       <c r="C61" s="6" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="D61" s="25" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.1216216216216216</v>
       </c>
     </row>
     <row r="62">
@@ -5796,11 +5796,11 @@
           <t>B.Ed</t>
         </is>
       </c>
-      <c r="C62" s="9" t="n">
-        <v>0</v>
+      <c r="C62" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="D62" s="25" t="n">
-        <v>0</v>
+        <v>0.01351351351351351</v>
       </c>
     </row>
     <row r="63">
@@ -5848,10 +5848,10 @@
         </is>
       </c>
       <c r="C66" s="6" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="D66" s="25" t="n">
-        <v>0.3928571428571428</v>
+        <v>0.4054054054054054</v>
       </c>
     </row>
     <row r="67">
@@ -5861,10 +5861,10 @@
         </is>
       </c>
       <c r="C67" s="6" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="D67" s="25" t="n">
-        <v>0.4642857142857143</v>
+        <v>0.4864864864864865</v>
       </c>
     </row>
     <row r="68">
@@ -5874,10 +5874,10 @@
         </is>
       </c>
       <c r="C68" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D68" s="25" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.06756756756756757</v>
       </c>
     </row>
     <row r="69">
@@ -5890,7 +5890,7 @@
         <v>1</v>
       </c>
       <c r="D69" s="25" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.01351351351351351</v>
       </c>
     </row>
     <row r="70">
@@ -5900,10 +5900,10 @@
         </is>
       </c>
       <c r="C70" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D70" s="25" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.02702702702702703</v>
       </c>
     </row>
     <row r="71">
@@ -5954,7 +5954,7 @@
         <v>2</v>
       </c>
       <c r="D74" s="25" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.02702702702702703</v>
       </c>
     </row>
     <row r="75">
@@ -5964,10 +5964,10 @@
         </is>
       </c>
       <c r="C75" s="6" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D75" s="25" t="n">
-        <v>0.5892857142857143</v>
+        <v>0.4324324324324325</v>
       </c>
     </row>
     <row r="76">
@@ -5980,7 +5980,7 @@
         <v>14</v>
       </c>
       <c r="D76" s="25" t="n">
-        <v>0.25</v>
+        <v>0.1891891891891892</v>
       </c>
     </row>
     <row r="77">
@@ -5993,7 +5993,7 @@
         <v>4</v>
       </c>
       <c r="D77" s="25" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.05405405405405406</v>
       </c>
     </row>
     <row r="78">
@@ -6006,7 +6006,7 @@
         <v>1</v>
       </c>
       <c r="D78" s="25" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.01351351351351351</v>
       </c>
     </row>
     <row r="79">
@@ -6083,7 +6083,7 @@
         <v>4</v>
       </c>
       <c r="D84" s="25" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.05405405405405406</v>
       </c>
     </row>
     <row r="85">
@@ -6096,7 +6096,7 @@
         <v>9</v>
       </c>
       <c r="D85" s="25" t="n">
-        <v>0.1607142857142857</v>
+        <v>0.1216216216216216</v>
       </c>
     </row>
     <row r="86">
@@ -6106,10 +6106,10 @@
         </is>
       </c>
       <c r="C86" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D86" s="25" t="n">
-        <v>0.05357142857142857</v>
+        <v>0.06756756756756757</v>
       </c>
     </row>
     <row r="87">
@@ -6119,10 +6119,10 @@
         </is>
       </c>
       <c r="C87" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D87" s="25" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.0945945945945946</v>
       </c>
     </row>
     <row r="88">
@@ -6132,10 +6132,10 @@
         </is>
       </c>
       <c r="C88" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D88" s="25" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.05405405405405406</v>
       </c>
     </row>
     <row r="89">
@@ -6148,7 +6148,7 @@
         <v>2</v>
       </c>
       <c r="D89" s="25" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.02702702702702703</v>
       </c>
     </row>
     <row r="90">
@@ -6161,7 +6161,7 @@
         <v>1</v>
       </c>
       <c r="D90" s="25" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.01351351351351351</v>
       </c>
     </row>
     <row r="91">
@@ -6171,10 +6171,10 @@
         </is>
       </c>
       <c r="C91" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D91" s="25" t="n">
-        <v>0.1071428571428571</v>
+        <v>0.1081081081081081</v>
       </c>
     </row>
     <row r="92">
@@ -6184,10 +6184,10 @@
         </is>
       </c>
       <c r="C92" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D92" s="25" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.1351351351351351</v>
       </c>
     </row>
     <row r="93">
@@ -6197,10 +6197,10 @@
         </is>
       </c>
       <c r="C93" s="6" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D93" s="25" t="n">
-        <v>0.2678571428571428</v>
+        <v>0.3108108108108108</v>
       </c>
     </row>
     <row r="94">
@@ -6251,7 +6251,7 @@
         <v>40</v>
       </c>
       <c r="D97" s="25" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.5405405405405406</v>
       </c>
     </row>
     <row r="98">
@@ -6264,7 +6264,7 @@
         <v>25</v>
       </c>
       <c r="D98" s="25" t="n">
-        <v>0.4464285714285715</v>
+        <v>0.3378378378378378</v>
       </c>
     </row>
     <row r="99">
@@ -6277,7 +6277,7 @@
         <v>46</v>
       </c>
       <c r="D99" s="25" t="n">
-        <v>0.8214285714285714</v>
+        <v>0.6216216216216216</v>
       </c>
     </row>
     <row r="100">
@@ -6316,7 +6316,7 @@
         <v>24</v>
       </c>
       <c r="D102" s="25" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.3243243243243243</v>
       </c>
     </row>
     <row r="103">
@@ -6342,7 +6342,7 @@
         <v>42</v>
       </c>
       <c r="D104" s="25" t="n">
-        <v>0.75</v>
+        <v>0.5675675675675675</v>
       </c>
     </row>
     <row r="105">
@@ -6355,7 +6355,7 @@
         <v>42</v>
       </c>
       <c r="D105" s="25" t="n">
-        <v>0.75</v>
+        <v>0.5675675675675675</v>
       </c>
     </row>
     <row r="106">
@@ -6368,7 +6368,7 @@
         <v>12</v>
       </c>
       <c r="D106" s="25" t="n">
-        <v>0.2142857142857143</v>
+        <v>0.1621621621621622</v>
       </c>
     </row>
     <row r="107">
@@ -6381,7 +6381,7 @@
         <v>5</v>
       </c>
       <c r="D107" s="25" t="n">
-        <v>0.08928571428571429</v>
+        <v>0.06756756756756757</v>
       </c>
     </row>
     <row r="108">
@@ -6407,7 +6407,7 @@
         <v>1</v>
       </c>
       <c r="D109" s="25" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.01351351351351351</v>
       </c>
     </row>
     <row r="110">
@@ -6420,7 +6420,7 @@
         <v>1</v>
       </c>
       <c r="D110" s="25" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.01351351351351351</v>
       </c>
     </row>
     <row r="111">
@@ -6471,7 +6471,7 @@
         <v>39</v>
       </c>
       <c r="D114" s="25" t="n">
-        <v>0.6964285714285714</v>
+        <v>0.527027027027027</v>
       </c>
     </row>
     <row r="115">
@@ -6484,7 +6484,7 @@
         <v>13</v>
       </c>
       <c r="D115" s="25" t="n">
-        <v>0.2321428571428572</v>
+        <v>0.1756756756756757</v>
       </c>
     </row>
     <row r="116">
@@ -6497,7 +6497,7 @@
         <v>16</v>
       </c>
       <c r="D116" s="25" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2162162162162162</v>
       </c>
     </row>
     <row r="117">
@@ -6510,7 +6510,7 @@
         <v>6</v>
       </c>
       <c r="D117" s="25" t="n">
-        <v>0.1071428571428571</v>
+        <v>0.08108108108108109</v>
       </c>
     </row>
     <row r="118">
@@ -6523,7 +6523,7 @@
         <v>7</v>
       </c>
       <c r="D118" s="25" t="n">
-        <v>0.125</v>
+        <v>0.0945945945945946</v>
       </c>
     </row>
     <row r="119">
@@ -6536,7 +6536,7 @@
         <v>21</v>
       </c>
       <c r="D119" s="25" t="n">
-        <v>0.375</v>
+        <v>0.2837837837837838</v>
       </c>
     </row>
     <row r="120">
@@ -6549,7 +6549,7 @@
         <v>5</v>
       </c>
       <c r="D120" s="25" t="n">
-        <v>0.08928571428571429</v>
+        <v>0.06756756756756757</v>
       </c>
     </row>
     <row r="121">
@@ -6562,7 +6562,7 @@
         <v>2</v>
       </c>
       <c r="D121" s="25" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.02702702702702703</v>
       </c>
     </row>
     <row r="122">
@@ -6575,7 +6575,7 @@
         <v>2</v>
       </c>
       <c r="D122" s="25" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.02702702702702703</v>
       </c>
     </row>
     <row r="123">
@@ -6588,7 +6588,7 @@
         <v>6</v>
       </c>
       <c r="D123" s="25" t="n">
-        <v>0.1071428571428571</v>
+        <v>0.08108108108108109</v>
       </c>
     </row>
     <row r="124">
@@ -6601,7 +6601,7 @@
         <v>36</v>
       </c>
       <c r="D124" s="25" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.4864864864864865</v>
       </c>
     </row>
     <row r="125">
@@ -6649,10 +6649,10 @@
         </is>
       </c>
       <c r="C128" s="6" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="D128" s="25" t="n">
-        <v>0.3571428571428572</v>
+        <v>0.3648648648648649</v>
       </c>
     </row>
     <row r="129">
@@ -6662,10 +6662,10 @@
         </is>
       </c>
       <c r="C129" s="6" t="n">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="D129" s="25" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.581081081081081</v>
       </c>
     </row>
     <row r="130">
@@ -6675,10 +6675,10 @@
         </is>
       </c>
       <c r="C130" s="6" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="D130" s="25" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.5405405405405406</v>
       </c>
     </row>
     <row r="131">
@@ -6701,10 +6701,10 @@
         </is>
       </c>
       <c r="C132" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D132" s="25" t="n">
-        <v>0.1785714285714286</v>
+        <v>0.1486486486486487</v>
       </c>
     </row>
     <row r="133">
@@ -6717,7 +6717,7 @@
         <v>1</v>
       </c>
       <c r="D133" s="25" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.01351351351351351</v>
       </c>
     </row>
     <row r="134">
@@ -6727,10 +6727,10 @@
         </is>
       </c>
       <c r="C134" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D134" s="25" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.04054054054054054</v>
       </c>
     </row>
     <row r="135">
@@ -6781,7 +6781,7 @@
         <v>26</v>
       </c>
       <c r="D138" s="25" t="n">
-        <v>0.4642857142857143</v>
+        <v>0.3513513513513514</v>
       </c>
     </row>
     <row r="139">
@@ -6794,7 +6794,7 @@
         <v>22</v>
       </c>
       <c r="D139" s="25" t="n">
-        <v>0.3928571428571428</v>
+        <v>0.2972972972972973</v>
       </c>
     </row>
     <row r="140">
@@ -6807,7 +6807,7 @@
         <v>27</v>
       </c>
       <c r="D140" s="25" t="n">
-        <v>0.4821428571428572</v>
+        <v>0.3648648648648649</v>
       </c>
     </row>
     <row r="141">
@@ -6820,7 +6820,7 @@
         <v>14</v>
       </c>
       <c r="D141" s="25" t="n">
-        <v>0.25</v>
+        <v>0.1891891891891892</v>
       </c>
     </row>
     <row r="142">
@@ -6833,7 +6833,7 @@
         <v>11</v>
       </c>
       <c r="D142" s="25" t="n">
-        <v>0.1964285714285714</v>
+        <v>0.1486486486486487</v>
       </c>
     </row>
     <row r="143">
@@ -6846,7 +6846,7 @@
         <v>14</v>
       </c>
       <c r="D143" s="25" t="n">
-        <v>0.25</v>
+        <v>0.1891891891891892</v>
       </c>
     </row>
     <row r="144">
@@ -6859,7 +6859,7 @@
         <v>17</v>
       </c>
       <c r="D144" s="25" t="n">
-        <v>0.3035714285714285</v>
+        <v>0.2297297297297297</v>
       </c>
     </row>
     <row r="145">
@@ -6907,10 +6907,10 @@
         </is>
       </c>
       <c r="C148" s="6" t="n">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="D148" s="25" t="n">
-        <v>0.625</v>
+        <v>0.6351351351351351</v>
       </c>
     </row>
     <row r="149">
@@ -6920,10 +6920,10 @@
         </is>
       </c>
       <c r="C149" s="6" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D149" s="25" t="n">
-        <v>0.2678571428571428</v>
+        <v>0.2837837837837838</v>
       </c>
     </row>
     <row r="150">
@@ -6933,10 +6933,10 @@
         </is>
       </c>
       <c r="C150" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D150" s="25" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.05405405405405406</v>
       </c>
     </row>
     <row r="151">
@@ -6945,11 +6945,11 @@
           <t>Rs 5,00,001-Rs 7,00,000</t>
         </is>
       </c>
-      <c r="C151" s="9" t="n">
-        <v>0</v>
+      <c r="C151" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="D151" s="25" t="n">
-        <v>0</v>
+        <v>0.01351351351351351</v>
       </c>
     </row>
     <row r="152">
@@ -7023,10 +7023,10 @@
         </is>
       </c>
       <c r="C157" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D157" s="25" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.04054054054054054</v>
       </c>
     </row>
     <row r="158">
@@ -7036,10 +7036,10 @@
         </is>
       </c>
       <c r="C158" s="6" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="D158" s="25" t="n">
-        <v>0.8928571428571429</v>
+        <v>0.9459459459459459</v>
       </c>
     </row>
     <row r="159">
@@ -7087,10 +7087,10 @@
         </is>
       </c>
       <c r="C162" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D162" s="25" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.04054054054054054</v>
       </c>
     </row>
     <row r="163">
@@ -7103,7 +7103,7 @@
         <v>1</v>
       </c>
       <c r="D163" s="25" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.01351351351351351</v>
       </c>
     </row>
     <row r="164">
@@ -7154,7 +7154,7 @@
         <v>1</v>
       </c>
       <c r="D167" s="25" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.01351351351351351</v>
       </c>
     </row>
     <row r="168">
@@ -7167,7 +7167,7 @@
         <v>5</v>
       </c>
       <c r="D168" s="25" t="n">
-        <v>0.08928571428571429</v>
+        <v>0.06756756756756757</v>
       </c>
     </row>
     <row r="169">
@@ -7190,10 +7190,10 @@
         </is>
       </c>
       <c r="C170" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D170" s="25" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.04054054054054054</v>
       </c>
     </row>
     <row r="171">
@@ -7216,10 +7216,10 @@
         </is>
       </c>
       <c r="C172" s="6" t="n">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="D172" s="25" t="n">
-        <v>0.75</v>
+        <v>0.8243243243243243</v>
       </c>
     </row>
     <row r="173">
@@ -7229,10 +7229,10 @@
         </is>
       </c>
       <c r="C173" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D173" s="25" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.04054054054054054</v>
       </c>
     </row>
     <row r="174">
@@ -7283,7 +7283,7 @@
         <v>1</v>
       </c>
       <c r="D177" s="25" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.01351351351351351</v>
       </c>
     </row>
     <row r="178">
@@ -7293,10 +7293,10 @@
         </is>
       </c>
       <c r="C178" s="6" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="D178" s="25" t="n">
-        <v>0.5714285714285714</v>
+        <v>0.6081081081081081</v>
       </c>
     </row>
     <row r="179">
@@ -7306,10 +7306,10 @@
         </is>
       </c>
       <c r="C179" s="6" t="n">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="D179" s="25" t="n">
-        <v>0.4464285714285715</v>
+        <v>0.5135135135135135</v>
       </c>
     </row>
     <row r="180">
@@ -7319,10 +7319,10 @@
         </is>
       </c>
       <c r="C180" s="6" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="D180" s="25" t="n">
-        <v>0.5178571428571429</v>
+        <v>0.5675675675675675</v>
       </c>
     </row>
     <row r="181">
@@ -7332,10 +7332,10 @@
         </is>
       </c>
       <c r="C181" s="6" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D181" s="25" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2567567567567567</v>
       </c>
     </row>
     <row r="182">
@@ -7348,7 +7348,7 @@
         <v>11</v>
       </c>
       <c r="D182" s="25" t="n">
-        <v>0.1964285714285714</v>
+        <v>0.1486486486486487</v>
       </c>
     </row>
     <row r="183">
@@ -7358,10 +7358,10 @@
         </is>
       </c>
       <c r="C183" s="6" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="D183" s="25" t="n">
-        <v>0.4464285714285715</v>
+        <v>0.4594594594594595</v>
       </c>
     </row>
     <row r="184">
@@ -7371,10 +7371,10 @@
         </is>
       </c>
       <c r="C184" s="6" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D184" s="25" t="n">
-        <v>0.125</v>
+        <v>0.1351351351351351</v>
       </c>
     </row>
     <row r="185">
@@ -7387,7 +7387,7 @@
         <v>4</v>
       </c>
       <c r="D185" s="25" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.05405405405405406</v>
       </c>
     </row>
     <row r="186">
@@ -7397,10 +7397,10 @@
         </is>
       </c>
       <c r="C186" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D186" s="25" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.06756756756756757</v>
       </c>
     </row>
     <row r="187">
@@ -7448,10 +7448,10 @@
         </is>
       </c>
       <c r="C190" s="6" t="n">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="D190" s="25" t="n">
-        <v>0.6607142857142857</v>
+        <v>0.7432432432432432</v>
       </c>
     </row>
     <row r="191">
@@ -7461,10 +7461,10 @@
         </is>
       </c>
       <c r="C191" s="6" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D191" s="25" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2432432432432433</v>
       </c>
     </row>
     <row r="192">
@@ -7474,10 +7474,10 @@
         </is>
       </c>
       <c r="C192" s="6" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D192" s="25" t="n">
-        <v>0.2678571428571428</v>
+        <v>0.2972972972972973</v>
       </c>
     </row>
     <row r="193">
@@ -7487,10 +7487,10 @@
         </is>
       </c>
       <c r="C193" s="6" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D193" s="25" t="n">
-        <v>0.2678571428571428</v>
+        <v>0.2702702702702703</v>
       </c>
     </row>
     <row r="194">
@@ -7503,7 +7503,7 @@
         <v>3</v>
       </c>
       <c r="D194" s="25" t="n">
-        <v>0.05357142857142857</v>
+        <v>0.04054054054054054</v>
       </c>
     </row>
     <row r="195">
@@ -7513,10 +7513,10 @@
         </is>
       </c>
       <c r="C195" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D195" s="25" t="n">
-        <v>0.08928571428571429</v>
+        <v>0.08108108108108109</v>
       </c>
     </row>
     <row r="196">
@@ -7529,7 +7529,7 @@
         <v>8</v>
       </c>
       <c r="D196" s="25" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.1081081081081081</v>
       </c>
     </row>
     <row r="197">
@@ -7539,10 +7539,10 @@
         </is>
       </c>
       <c r="C197" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D197" s="25" t="n">
-        <v>0.125</v>
+        <v>0.1216216216216216</v>
       </c>
     </row>
     <row r="198">
@@ -7590,10 +7590,10 @@
         </is>
       </c>
       <c r="C201" s="6" t="n">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="D201" s="25" t="n">
-        <v>0.5357142857142857</v>
+        <v>0.581081081081081</v>
       </c>
     </row>
     <row r="202">
@@ -7603,10 +7603,10 @@
         </is>
       </c>
       <c r="C202" s="6" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="D202" s="25" t="n">
-        <v>0.2142857142857143</v>
+        <v>0.2567567567567567</v>
       </c>
     </row>
     <row r="203">
@@ -7616,10 +7616,10 @@
         </is>
       </c>
       <c r="C203" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D203" s="25" t="n">
-        <v>0.1785714285714286</v>
+        <v>0.1486486486486487</v>
       </c>
     </row>
     <row r="204">
@@ -7667,10 +7667,10 @@
         </is>
       </c>
       <c r="C207" s="6" t="n">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="D207" s="25" t="n">
-        <v>0.5535714285714286</v>
+        <v>0.6351351351351351</v>
       </c>
     </row>
     <row r="208">
@@ -7680,10 +7680,10 @@
         </is>
       </c>
       <c r="C208" s="6" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D208" s="25" t="n">
-        <v>0.375</v>
+        <v>0.3513513513513514</v>
       </c>
     </row>
     <row r="209">
@@ -7731,10 +7731,10 @@
         </is>
       </c>
       <c r="C212" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D212" s="25" t="n">
-        <v>0.1071428571428571</v>
+        <v>0.1081081081081081</v>
       </c>
     </row>
     <row r="213">
@@ -7744,10 +7744,10 @@
         </is>
       </c>
       <c r="C213" s="6" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="D213" s="25" t="n">
-        <v>0.2321428571428572</v>
+        <v>0.2837837837837838</v>
       </c>
     </row>
     <row r="214">
@@ -7757,10 +7757,10 @@
         </is>
       </c>
       <c r="C214" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D214" s="25" t="n">
-        <v>0.1607142857142857</v>
+        <v>0.1621621621621622</v>
       </c>
     </row>
     <row r="215">
@@ -7770,10 +7770,10 @@
         </is>
       </c>
       <c r="C215" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D215" s="25" t="n">
-        <v>0.05357142857142857</v>
+        <v>0.05405405405405406</v>
       </c>
     </row>
     <row r="216">
@@ -7782,11 +7782,11 @@
           <t>More than 40</t>
         </is>
       </c>
-      <c r="C216" s="9" t="n">
-        <v>0</v>
+      <c r="C216" s="6" t="n">
+        <v>2</v>
       </c>
       <c r="D216" s="25" t="n">
-        <v>0</v>
+        <v>0.02702702702702703</v>
       </c>
     </row>
     <row r="217">
@@ -7834,10 +7834,10 @@
         </is>
       </c>
       <c r="C220" s="6" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="D220" s="25" t="n">
-        <v>0.2142857142857143</v>
+        <v>0.2567567567567567</v>
       </c>
     </row>
     <row r="221">
@@ -7850,7 +7850,7 @@
         <v>1</v>
       </c>
       <c r="D221" s="25" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.01351351351351351</v>
       </c>
     </row>
     <row r="222">
@@ -7860,10 +7860,10 @@
         </is>
       </c>
       <c r="C222" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D222" s="25" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.04054054054054054</v>
       </c>
     </row>
     <row r="223">
@@ -7876,7 +7876,7 @@
         <v>4</v>
       </c>
       <c r="D223" s="25" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.05405405405405406</v>
       </c>
     </row>
     <row r="224">
@@ -7889,7 +7889,7 @@
         <v>3</v>
       </c>
       <c r="D224" s="25" t="n">
-        <v>0.05357142857142857</v>
+        <v>0.04054054054054054</v>
       </c>
     </row>
     <row r="225">
@@ -7899,10 +7899,10 @@
         </is>
       </c>
       <c r="C225" s="6" t="n">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="D225" s="25" t="n">
-        <v>0.375</v>
+        <v>0.3918918918918919</v>
       </c>
     </row>
     <row r="226">
@@ -7912,10 +7912,10 @@
         </is>
       </c>
       <c r="C226" s="6" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D226" s="25" t="n">
-        <v>0.1607142857142857</v>
+        <v>0.1891891891891892</v>
       </c>
     </row>
     <row r="227">
@@ -7963,10 +7963,10 @@
         </is>
       </c>
       <c r="C230" s="6" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="D230" s="25" t="n">
-        <v>0.25</v>
+        <v>0.2837837837837838</v>
       </c>
     </row>
     <row r="231">
@@ -7976,10 +7976,10 @@
         </is>
       </c>
       <c r="C231" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D231" s="25" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.05405405405405406</v>
       </c>
     </row>
     <row r="232">
@@ -8001,11 +8001,11 @@
           <t>Facebook</t>
         </is>
       </c>
-      <c r="C233" s="9" t="n">
-        <v>0</v>
+      <c r="C233" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="D233" s="25" t="n">
-        <v>0</v>
+        <v>0.01351351351351351</v>
       </c>
     </row>
     <row r="234">
@@ -8028,10 +8028,10 @@
         </is>
       </c>
       <c r="C235" s="6" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="D235" s="25" t="n">
-        <v>0.7142857142857143</v>
+        <v>0.7432432432432432</v>
       </c>
     </row>
     <row r="236">
@@ -8079,10 +8079,10 @@
         </is>
       </c>
       <c r="C239" s="6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D239" s="25" t="n">
-        <v>0.125</v>
+        <v>0.1486486486486487</v>
       </c>
     </row>
     <row r="240">
@@ -8092,10 +8092,10 @@
         </is>
       </c>
       <c r="C240" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D240" s="25" t="n">
-        <v>0.1607142857142857</v>
+        <v>0.1621621621621622</v>
       </c>
     </row>
     <row r="241">
@@ -8108,7 +8108,7 @@
         <v>4</v>
       </c>
       <c r="D241" s="25" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.05405405405405406</v>
       </c>
     </row>
     <row r="242">
@@ -8121,7 +8121,7 @@
         <v>5</v>
       </c>
       <c r="D242" s="25" t="n">
-        <v>0.08928571428571429</v>
+        <v>0.06756756756756757</v>
       </c>
     </row>
     <row r="243">
@@ -8178,7 +8178,7 @@
       </c>
       <c r="C247" s="32" t="inlineStr">
         <is>
-          <t>3.8 Years</t>
+          <t>4.0 Years</t>
         </is>
       </c>
     </row>
@@ -8190,7 +8190,7 @@
       </c>
       <c r="C248" s="32" t="inlineStr">
         <is>
-          <t>3.0 Years</t>
+          <t>3.2 Years</t>
         </is>
       </c>
     </row>
@@ -8202,7 +8202,7 @@
       </c>
       <c r="C249" s="32" t="inlineStr">
         <is>
-          <t>4.6 Years</t>
+          <t>4.7 Years</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Dausa 1:1 primary activity mapping: balance Social Category Matrix and Finance counts to exact N=50
</commit_message>
<xml_diff>
--- a/Projects/CmF_SHG_Women_Entrepreneurs/reports/district_analysis/All_Rajasthan/excel/All_Rajasthan_Survey_Analysis_Master.xlsx
+++ b/Projects/CmF_SHG_Women_Entrepreneurs/reports/district_analysis/All_Rajasthan/excel/All_Rajasthan_Survey_Analysis_Master.xlsx
@@ -816,22 +816,22 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>2563000</v>
+        <v>1931000</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>183071.4285714286</v>
+        <v>160916.6666666667</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>285000</v>
+        <v>205000</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>205000</v>
+        <v>180000</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>1184000</v>
+        <v>774000</v>
       </c>
       <c r="J4" s="8" t="n">
         <v>0</v>
@@ -840,16 +840,16 @@
         <v>0</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="M4" s="8" t="n">
         <v>0</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>319000</v>
+        <v>262000</v>
       </c>
       <c r="O4" s="7" t="n">
-        <v>360000</v>
+        <v>320000</v>
       </c>
       <c r="P4" s="7" t="n">
         <v>80000</v>
@@ -867,7 +867,7 @@
         <v>0</v>
       </c>
       <c r="U4" s="6" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -946,22 +946,22 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>483000</v>
+        <v>4</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>80500</v>
-      </c>
-      <c r="G6" s="7" t="n">
-        <v>92000</v>
+        <v>0</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="H6" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="7" t="n">
-        <v>231000</v>
+      <c r="I6" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="J6" s="8" t="n">
         <v>0</v>
@@ -975,11 +975,11 @@
       <c r="M6" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="N6" s="7" t="n">
-        <v>90000</v>
-      </c>
-      <c r="O6" s="7" t="n">
-        <v>70000</v>
+      <c r="N6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="P6" s="8" t="n">
         <v>0</v>
@@ -996,8 +996,8 @@
       <c r="T6" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="U6" s="6" t="n">
-        <v>2</v>
+      <c r="U6" s="9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -1490,13 +1490,13 @@
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E14" s="7" t="n">
         <v>3862501</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>203289.5263157895</v>
+        <v>214583.3888888889</v>
       </c>
       <c r="G14" s="7" t="n">
         <v>1523501</v>
@@ -3883,7 +3883,7 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>1</v>
@@ -3892,10 +3892,10 @@
         <v>4</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -3941,13 +3941,13 @@
         <v>0</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="6" t="n">
         <v>4</v>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -4163,10 +4163,10 @@
         <v>9</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16">

</xml_diff>

<commit_message>
Ingest Baran district survey responses and update multi-district analysis engine
</commit_message>
<xml_diff>
--- a/Projects/CmF_SHG_Women_Entrepreneurs/reports/district_analysis/All_Rajasthan/excel/All_Rajasthan_Survey_Analysis_Master.xlsx
+++ b/Projects/CmF_SHG_Women_Entrepreneurs/reports/district_analysis/All_Rajasthan/excel/All_Rajasthan_Survey_Analysis_Master.xlsx
@@ -751,13 +751,13 @@
         </is>
       </c>
       <c r="D3" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3" s="7" t="n">
         <v>880000</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>440000</v>
+        <v>293333.3333333333</v>
       </c>
       <c r="G3" s="7" t="n">
         <v>215000</v>
@@ -816,13 +816,13 @@
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>1931000</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>160916.6666666667</v>
+        <v>128733.3333333333</v>
       </c>
       <c r="G4" s="7" t="n">
         <v>205000</v>
@@ -881,13 +881,13 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E5" s="7" t="n">
         <v>2703000</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>245727.2727272727</v>
+        <v>193071.4285714286</v>
       </c>
       <c r="G5" s="7" t="n">
         <v>520000</v>
@@ -946,7 +946,7 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E6" s="8" t="n">
         <v>0</v>
@@ -1425,13 +1425,13 @@
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E13" s="7" t="n">
         <v>286500</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>71625</v>
+        <v>57300</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>55000</v>
@@ -1685,13 +1685,13 @@
         </is>
       </c>
       <c r="D17" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E17" s="7" t="n">
         <v>470000</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>470000</v>
+        <v>156666.6666666667</v>
       </c>
       <c r="G17" s="7" t="n">
         <v>68000</v>
@@ -2164,13 +2164,13 @@
         </is>
       </c>
       <c r="D24" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E24" s="7" t="n">
         <v>568500</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>189500</v>
+        <v>142125</v>
       </c>
       <c r="G24" s="7" t="n">
         <v>77500</v>
@@ -2229,13 +2229,13 @@
         </is>
       </c>
       <c r="D25" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E25" s="7" t="n">
         <v>62300</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>31150</v>
+        <v>15575</v>
       </c>
       <c r="G25" s="7" t="n">
         <v>17000</v>
@@ -2424,13 +2424,13 @@
         </is>
       </c>
       <c r="D28" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E28" s="7" t="n">
         <v>1033601</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>206720.2</v>
+        <v>172266.8333333333</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>270000</v>
@@ -3863,13 +3863,13 @@
         <v>0</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4" s="6" t="n">
         <v>1</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -3889,13 +3889,13 @@
         <v>1</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G5" s="6" t="n">
         <v>2</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -3915,13 +3915,13 @@
         <v>1</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
@@ -3941,13 +3941,13 @@
         <v>0</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G7" s="6" t="n">
         <v>3</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -4133,14 +4133,14 @@
       <c r="E14" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="9" t="n">
-        <v>0</v>
+      <c r="F14" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="G14" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -4232,19 +4232,19 @@
         </is>
       </c>
       <c r="D18" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="9" t="n">
-        <v>0</v>
-      </c>
       <c r="G18" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
@@ -4431,13 +4431,13 @@
         <v>1</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G25" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26">
@@ -4451,19 +4451,19 @@
         </is>
       </c>
       <c r="D26" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" s="9" t="n">
         <v>0</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G26" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27">
@@ -4535,13 +4535,13 @@
         <v>0</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G29" s="6" t="n">
         <v>1</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30">
@@ -4801,10 +4801,10 @@
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="D4" s="25" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2777777777777778</v>
       </c>
     </row>
     <row r="5">
@@ -4814,10 +4814,10 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>0.2702702702702703</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="6">
@@ -4827,10 +4827,10 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>0.3108108108108108</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="7">
@@ -4840,10 +4840,10 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>0.3108108108108108</v>
+        <v>0.3666666666666666</v>
       </c>
     </row>
     <row r="8">
@@ -4853,10 +4853,10 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D8" s="25" t="n">
-        <v>0.3648648648648649</v>
+        <v>0.3222222222222222</v>
       </c>
     </row>
     <row r="9">
@@ -4905,10 +4905,10 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D13" s="25" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2555555555555555</v>
       </c>
     </row>
     <row r="14">
@@ -4918,10 +4918,10 @@
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D14" s="25" t="n">
-        <v>0.3108108108108108</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="15">
@@ -4931,10 +4931,10 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2333333333333333</v>
       </c>
     </row>
     <row r="16">
@@ -4960,7 +4960,7 @@
         <v>1</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>0.01351351351351351</v>
+        <v>0.01111111111111111</v>
       </c>
     </row>
     <row r="18">
@@ -4970,10 +4970,10 @@
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D18" s="25" t="n">
-        <v>0.2027027027027027</v>
+        <v>0.1777777777777778</v>
       </c>
     </row>
     <row r="19">
@@ -5030,7 +5030,7 @@
         </is>
       </c>
       <c r="C2" s="27" t="n">
-        <v>74</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3"/>
@@ -5063,10 +5063,10 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>0.6351351351351351</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="6">
@@ -5076,10 +5076,10 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>0.3648648648648649</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="7">
@@ -5127,10 +5127,10 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2111111111111111</v>
       </c>
     </row>
     <row r="11">
@@ -5140,10 +5140,10 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="D11" s="25" t="n">
-        <v>0.7702702702702703</v>
+        <v>0.7888888888888889</v>
       </c>
     </row>
     <row r="12">
@@ -5191,10 +5191,10 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>0.4054054054054054</v>
+        <v>0.4444444444444444</v>
       </c>
     </row>
     <row r="16">
@@ -5204,10 +5204,10 @@
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D16" s="25" t="n">
-        <v>0.4324324324324325</v>
+        <v>0.3888888888888889</v>
       </c>
     </row>
     <row r="17">
@@ -5217,10 +5217,10 @@
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>0.2162162162162162</v>
+        <v>0.2333333333333333</v>
       </c>
     </row>
     <row r="18">
@@ -5268,10 +5268,10 @@
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="D21" s="25" t="n">
-        <v>0.9594594594594594</v>
+        <v>0.9666666666666667</v>
       </c>
     </row>
     <row r="22">
@@ -5281,7 +5281,7 @@
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>74</v>
+        <v>90</v>
       </c>
       <c r="D22" s="25" t="n">
         <v>1</v>
@@ -5294,10 +5294,10 @@
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>0.6351351351351351</v>
+        <v>0.6777777777777778</v>
       </c>
     </row>
     <row r="24">
@@ -5307,10 +5307,10 @@
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D24" s="25" t="n">
-        <v>0.05405405405405406</v>
+        <v>0.05555555555555555</v>
       </c>
     </row>
     <row r="25">
@@ -5323,7 +5323,7 @@
         <v>3</v>
       </c>
       <c r="D25" s="25" t="n">
-        <v>0.04054054054054054</v>
+        <v>0.03333333333333333</v>
       </c>
     </row>
     <row r="26">
@@ -5333,10 +5333,10 @@
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="D26" s="25" t="n">
-        <v>0.9459459459459459</v>
+        <v>0.8888888888888888</v>
       </c>
     </row>
     <row r="27">
@@ -5346,10 +5346,10 @@
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="D27" s="25" t="n">
-        <v>0.5405405405405406</v>
+        <v>0.5555555555555556</v>
       </c>
     </row>
     <row r="28">
@@ -5400,7 +5400,7 @@
         <v>2</v>
       </c>
       <c r="D31" s="25" t="n">
-        <v>0.02702702702702703</v>
+        <v>0.02222222222222222</v>
       </c>
     </row>
     <row r="32">
@@ -5410,10 +5410,10 @@
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D32" s="25" t="n">
-        <v>0.4189189189189189</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="33">
@@ -5423,10 +5423,10 @@
         </is>
       </c>
       <c r="C33" s="6" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="D33" s="25" t="n">
-        <v>0.3783783783783784</v>
+        <v>0.4222222222222222</v>
       </c>
     </row>
     <row r="34">
@@ -5436,10 +5436,10 @@
         </is>
       </c>
       <c r="C34" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D34" s="25" t="n">
-        <v>0.1351351351351351</v>
+        <v>0.1222222222222222</v>
       </c>
     </row>
     <row r="35">
@@ -5452,7 +5452,7 @@
         <v>3</v>
       </c>
       <c r="D35" s="25" t="n">
-        <v>0.04054054054054054</v>
+        <v>0.03333333333333333</v>
       </c>
     </row>
     <row r="36">
@@ -5513,10 +5513,10 @@
         </is>
       </c>
       <c r="C40" s="6" t="n">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="D40" s="25" t="n">
-        <v>0.9459459459459459</v>
+        <v>0.9555555555555556</v>
       </c>
     </row>
     <row r="41">
@@ -5529,7 +5529,7 @@
         <v>4</v>
       </c>
       <c r="D41" s="25" t="n">
-        <v>0.05405405405405406</v>
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="42">
@@ -5603,10 +5603,10 @@
         </is>
       </c>
       <c r="C47" s="6" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D47" s="25" t="n">
-        <v>0.3378378378378378</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="48">
@@ -5619,7 +5619,7 @@
         <v>4</v>
       </c>
       <c r="D48" s="25" t="n">
-        <v>0.05405405405405406</v>
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="49">
@@ -5629,10 +5629,10 @@
         </is>
       </c>
       <c r="C49" s="6" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="D49" s="25" t="n">
-        <v>0.3783783783783784</v>
+        <v>0.4555555555555555</v>
       </c>
     </row>
     <row r="50">
@@ -5642,10 +5642,10 @@
         </is>
       </c>
       <c r="C50" s="6" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D50" s="25" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="51">
@@ -5693,10 +5693,10 @@
         </is>
       </c>
       <c r="C54" s="6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D54" s="25" t="n">
-        <v>0.1216216216216216</v>
+        <v>0.1111111111111111</v>
       </c>
     </row>
     <row r="55">
@@ -5706,10 +5706,10 @@
         </is>
       </c>
       <c r="C55" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D55" s="25" t="n">
-        <v>0.01351351351351351</v>
+        <v>0.02222222222222222</v>
       </c>
     </row>
     <row r="56">
@@ -5719,10 +5719,10 @@
         </is>
       </c>
       <c r="C56" s="6" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D56" s="25" t="n">
-        <v>0.2432432432432433</v>
+        <v>0.2111111111111111</v>
       </c>
     </row>
     <row r="57">
@@ -5732,10 +5732,10 @@
         </is>
       </c>
       <c r="C57" s="6" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D57" s="25" t="n">
-        <v>0.1486486486486487</v>
+        <v>0.1555555555555556</v>
       </c>
     </row>
     <row r="58">
@@ -5745,10 +5745,10 @@
         </is>
       </c>
       <c r="C58" s="6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D58" s="25" t="n">
-        <v>0.1891891891891892</v>
+        <v>0.1666666666666667</v>
       </c>
     </row>
     <row r="59">
@@ -5758,10 +5758,10 @@
         </is>
       </c>
       <c r="C59" s="6" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D59" s="25" t="n">
-        <v>0.1486486486486487</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="60">
@@ -5784,10 +5784,10 @@
         </is>
       </c>
       <c r="C61" s="6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D61" s="25" t="n">
-        <v>0.1216216216216216</v>
+        <v>0.1222222222222222</v>
       </c>
     </row>
     <row r="62">
@@ -5800,7 +5800,7 @@
         <v>1</v>
       </c>
       <c r="D62" s="25" t="n">
-        <v>0.01351351351351351</v>
+        <v>0.01111111111111111</v>
       </c>
     </row>
     <row r="63">
@@ -5848,10 +5848,10 @@
         </is>
       </c>
       <c r="C66" s="6" t="n">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D66" s="25" t="n">
-        <v>0.4054054054054054</v>
+        <v>0.4222222222222222</v>
       </c>
     </row>
     <row r="67">
@@ -5861,10 +5861,10 @@
         </is>
       </c>
       <c r="C67" s="6" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D67" s="25" t="n">
-        <v>0.4864864864864865</v>
+        <v>0.4666666666666667</v>
       </c>
     </row>
     <row r="68">
@@ -5874,10 +5874,10 @@
         </is>
       </c>
       <c r="C68" s="6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D68" s="25" t="n">
-        <v>0.06756756756756757</v>
+        <v>0.07777777777777778</v>
       </c>
     </row>
     <row r="69">
@@ -5890,7 +5890,7 @@
         <v>1</v>
       </c>
       <c r="D69" s="25" t="n">
-        <v>0.01351351351351351</v>
+        <v>0.01111111111111111</v>
       </c>
     </row>
     <row r="70">
@@ -5903,7 +5903,7 @@
         <v>2</v>
       </c>
       <c r="D70" s="25" t="n">
-        <v>0.02702702702702703</v>
+        <v>0.02222222222222222</v>
       </c>
     </row>
     <row r="71">
@@ -5954,7 +5954,7 @@
         <v>2</v>
       </c>
       <c r="D74" s="25" t="n">
-        <v>0.02702702702702703</v>
+        <v>0.02222222222222222</v>
       </c>
     </row>
     <row r="75">
@@ -5964,10 +5964,10 @@
         </is>
       </c>
       <c r="C75" s="6" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D75" s="25" t="n">
-        <v>0.4324324324324325</v>
+        <v>0.3888888888888889</v>
       </c>
     </row>
     <row r="76">
@@ -5980,7 +5980,7 @@
         <v>14</v>
       </c>
       <c r="D76" s="25" t="n">
-        <v>0.1891891891891892</v>
+        <v>0.1555555555555556</v>
       </c>
     </row>
     <row r="77">
@@ -5990,10 +5990,10 @@
         </is>
       </c>
       <c r="C77" s="6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D77" s="25" t="n">
-        <v>0.05405405405405406</v>
+        <v>0.07777777777777778</v>
       </c>
     </row>
     <row r="78">
@@ -6006,7 +6006,7 @@
         <v>1</v>
       </c>
       <c r="D78" s="25" t="n">
-        <v>0.01351351351351351</v>
+        <v>0.01111111111111111</v>
       </c>
     </row>
     <row r="79">
@@ -6083,7 +6083,7 @@
         <v>4</v>
       </c>
       <c r="D84" s="25" t="n">
-        <v>0.05405405405405406</v>
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="85">
@@ -6093,10 +6093,10 @@
         </is>
       </c>
       <c r="C85" s="6" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D85" s="25" t="n">
-        <v>0.1216216216216216</v>
+        <v>0.1222222222222222</v>
       </c>
     </row>
     <row r="86">
@@ -6109,7 +6109,7 @@
         <v>5</v>
       </c>
       <c r="D86" s="25" t="n">
-        <v>0.06756756756756757</v>
+        <v>0.05555555555555555</v>
       </c>
     </row>
     <row r="87">
@@ -6119,10 +6119,10 @@
         </is>
       </c>
       <c r="C87" s="6" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D87" s="25" t="n">
-        <v>0.0945945945945946</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="88">
@@ -6135,7 +6135,7 @@
         <v>4</v>
       </c>
       <c r="D88" s="25" t="n">
-        <v>0.05405405405405406</v>
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="89">
@@ -6148,7 +6148,7 @@
         <v>2</v>
       </c>
       <c r="D89" s="25" t="n">
-        <v>0.02702702702702703</v>
+        <v>0.02222222222222222</v>
       </c>
     </row>
     <row r="90">
@@ -6158,10 +6158,10 @@
         </is>
       </c>
       <c r="C90" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D90" s="25" t="n">
-        <v>0.01351351351351351</v>
+        <v>0.02222222222222222</v>
       </c>
     </row>
     <row r="91">
@@ -6171,10 +6171,10 @@
         </is>
       </c>
       <c r="C91" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D91" s="25" t="n">
-        <v>0.1081081081081081</v>
+        <v>0.1111111111111111</v>
       </c>
     </row>
     <row r="92">
@@ -6184,10 +6184,10 @@
         </is>
       </c>
       <c r="C92" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D92" s="25" t="n">
-        <v>0.1351351351351351</v>
+        <v>0.1222222222222222</v>
       </c>
     </row>
     <row r="93">
@@ -6197,10 +6197,10 @@
         </is>
       </c>
       <c r="C93" s="6" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="D93" s="25" t="n">
-        <v>0.3108108108108108</v>
+        <v>0.3444444444444444</v>
       </c>
     </row>
     <row r="94">
@@ -6251,7 +6251,7 @@
         <v>40</v>
       </c>
       <c r="D97" s="25" t="n">
-        <v>0.5405405405405406</v>
+        <v>0.4444444444444444</v>
       </c>
     </row>
     <row r="98">
@@ -6264,7 +6264,7 @@
         <v>25</v>
       </c>
       <c r="D98" s="25" t="n">
-        <v>0.3378378378378378</v>
+        <v>0.2777777777777778</v>
       </c>
     </row>
     <row r="99">
@@ -6277,7 +6277,7 @@
         <v>46</v>
       </c>
       <c r="D99" s="25" t="n">
-        <v>0.6216216216216216</v>
+        <v>0.5111111111111111</v>
       </c>
     </row>
     <row r="100">
@@ -6316,7 +6316,7 @@
         <v>24</v>
       </c>
       <c r="D102" s="25" t="n">
-        <v>0.3243243243243243</v>
+        <v>0.2666666666666667</v>
       </c>
     </row>
     <row r="103">
@@ -6342,7 +6342,7 @@
         <v>42</v>
       </c>
       <c r="D104" s="25" t="n">
-        <v>0.5675675675675675</v>
+        <v>0.4666666666666667</v>
       </c>
     </row>
     <row r="105">
@@ -6355,7 +6355,7 @@
         <v>42</v>
       </c>
       <c r="D105" s="25" t="n">
-        <v>0.5675675675675675</v>
+        <v>0.4666666666666667</v>
       </c>
     </row>
     <row r="106">
@@ -6368,7 +6368,7 @@
         <v>12</v>
       </c>
       <c r="D106" s="25" t="n">
-        <v>0.1621621621621622</v>
+        <v>0.1333333333333333</v>
       </c>
     </row>
     <row r="107">
@@ -6381,7 +6381,7 @@
         <v>5</v>
       </c>
       <c r="D107" s="25" t="n">
-        <v>0.06756756756756757</v>
+        <v>0.05555555555555555</v>
       </c>
     </row>
     <row r="108">
@@ -6407,7 +6407,7 @@
         <v>1</v>
       </c>
       <c r="D109" s="25" t="n">
-        <v>0.01351351351351351</v>
+        <v>0.01111111111111111</v>
       </c>
     </row>
     <row r="110">
@@ -6420,7 +6420,7 @@
         <v>1</v>
       </c>
       <c r="D110" s="25" t="n">
-        <v>0.01351351351351351</v>
+        <v>0.01111111111111111</v>
       </c>
     </row>
     <row r="111">
@@ -6471,7 +6471,7 @@
         <v>39</v>
       </c>
       <c r="D114" s="25" t="n">
-        <v>0.527027027027027</v>
+        <v>0.4333333333333333</v>
       </c>
     </row>
     <row r="115">
@@ -6484,7 +6484,7 @@
         <v>13</v>
       </c>
       <c r="D115" s="25" t="n">
-        <v>0.1756756756756757</v>
+        <v>0.1444444444444444</v>
       </c>
     </row>
     <row r="116">
@@ -6497,7 +6497,7 @@
         <v>16</v>
       </c>
       <c r="D116" s="25" t="n">
-        <v>0.2162162162162162</v>
+        <v>0.1777777777777778</v>
       </c>
     </row>
     <row r="117">
@@ -6510,7 +6510,7 @@
         <v>6</v>
       </c>
       <c r="D117" s="25" t="n">
-        <v>0.08108108108108109</v>
+        <v>0.06666666666666667</v>
       </c>
     </row>
     <row r="118">
@@ -6523,7 +6523,7 @@
         <v>7</v>
       </c>
       <c r="D118" s="25" t="n">
-        <v>0.0945945945945946</v>
+        <v>0.07777777777777778</v>
       </c>
     </row>
     <row r="119">
@@ -6536,7 +6536,7 @@
         <v>21</v>
       </c>
       <c r="D119" s="25" t="n">
-        <v>0.2837837837837838</v>
+        <v>0.2333333333333333</v>
       </c>
     </row>
     <row r="120">
@@ -6549,7 +6549,7 @@
         <v>5</v>
       </c>
       <c r="D120" s="25" t="n">
-        <v>0.06756756756756757</v>
+        <v>0.05555555555555555</v>
       </c>
     </row>
     <row r="121">
@@ -6562,7 +6562,7 @@
         <v>2</v>
       </c>
       <c r="D121" s="25" t="n">
-        <v>0.02702702702702703</v>
+        <v>0.02222222222222222</v>
       </c>
     </row>
     <row r="122">
@@ -6575,7 +6575,7 @@
         <v>2</v>
       </c>
       <c r="D122" s="25" t="n">
-        <v>0.02702702702702703</v>
+        <v>0.02222222222222222</v>
       </c>
     </row>
     <row r="123">
@@ -6588,7 +6588,7 @@
         <v>6</v>
       </c>
       <c r="D123" s="25" t="n">
-        <v>0.08108108108108109</v>
+        <v>0.06666666666666667</v>
       </c>
     </row>
     <row r="124">
@@ -6601,7 +6601,7 @@
         <v>36</v>
       </c>
       <c r="D124" s="25" t="n">
-        <v>0.4864864864864865</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="125">
@@ -6649,10 +6649,10 @@
         </is>
       </c>
       <c r="C128" s="6" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="D128" s="25" t="n">
-        <v>0.3648648648648649</v>
+        <v>0.4222222222222222</v>
       </c>
     </row>
     <row r="129">
@@ -6662,10 +6662,10 @@
         </is>
       </c>
       <c r="C129" s="6" t="n">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="D129" s="25" t="n">
-        <v>0.581081081081081</v>
+        <v>0.6222222222222222</v>
       </c>
     </row>
     <row r="130">
@@ -6675,10 +6675,10 @@
         </is>
       </c>
       <c r="C130" s="6" t="n">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D130" s="25" t="n">
-        <v>0.5405405405405406</v>
+        <v>0.4888888888888889</v>
       </c>
     </row>
     <row r="131">
@@ -6701,10 +6701,10 @@
         </is>
       </c>
       <c r="C132" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D132" s="25" t="n">
-        <v>0.1486486486486487</v>
+        <v>0.1444444444444444</v>
       </c>
     </row>
     <row r="133">
@@ -6717,7 +6717,7 @@
         <v>1</v>
       </c>
       <c r="D133" s="25" t="n">
-        <v>0.01351351351351351</v>
+        <v>0.01111111111111111</v>
       </c>
     </row>
     <row r="134">
@@ -6730,7 +6730,7 @@
         <v>3</v>
       </c>
       <c r="D134" s="25" t="n">
-        <v>0.04054054054054054</v>
+        <v>0.03333333333333333</v>
       </c>
     </row>
     <row r="135">
@@ -6778,10 +6778,10 @@
         </is>
       </c>
       <c r="C138" s="6" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D138" s="25" t="n">
-        <v>0.3513513513513514</v>
+        <v>0.3333333333333333</v>
       </c>
     </row>
     <row r="139">
@@ -6791,10 +6791,10 @@
         </is>
       </c>
       <c r="C139" s="6" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D139" s="25" t="n">
-        <v>0.2972972972972973</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="140">
@@ -6804,10 +6804,10 @@
         </is>
       </c>
       <c r="C140" s="6" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="D140" s="25" t="n">
-        <v>0.3648648648648649</v>
+        <v>0.3555555555555556</v>
       </c>
     </row>
     <row r="141">
@@ -6817,10 +6817,10 @@
         </is>
       </c>
       <c r="C141" s="6" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D141" s="25" t="n">
-        <v>0.1891891891891892</v>
+        <v>0.2111111111111111</v>
       </c>
     </row>
     <row r="142">
@@ -6830,10 +6830,10 @@
         </is>
       </c>
       <c r="C142" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D142" s="25" t="n">
-        <v>0.1486486486486487</v>
+        <v>0.1444444444444444</v>
       </c>
     </row>
     <row r="143">
@@ -6843,10 +6843,10 @@
         </is>
       </c>
       <c r="C143" s="6" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D143" s="25" t="n">
-        <v>0.1891891891891892</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="144">
@@ -6856,10 +6856,10 @@
         </is>
       </c>
       <c r="C144" s="6" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D144" s="25" t="n">
-        <v>0.2297297297297297</v>
+        <v>0.2444444444444444</v>
       </c>
     </row>
     <row r="145">
@@ -6907,10 +6907,10 @@
         </is>
       </c>
       <c r="C148" s="6" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="D148" s="25" t="n">
-        <v>0.6351351351351351</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="149">
@@ -6920,10 +6920,10 @@
         </is>
       </c>
       <c r="C149" s="6" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D149" s="25" t="n">
-        <v>0.2837837837837838</v>
+        <v>0.2888888888888889</v>
       </c>
     </row>
     <row r="150">
@@ -6933,10 +6933,10 @@
         </is>
       </c>
       <c r="C150" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D150" s="25" t="n">
-        <v>0.05405405405405406</v>
+        <v>0.05555555555555555</v>
       </c>
     </row>
     <row r="151">
@@ -6946,10 +6946,10 @@
         </is>
       </c>
       <c r="C151" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D151" s="25" t="n">
-        <v>0.01351351351351351</v>
+        <v>0.02222222222222222</v>
       </c>
     </row>
     <row r="152">
@@ -6971,11 +6971,11 @@
           <t>More than 9,00,000</t>
         </is>
       </c>
-      <c r="C153" s="9" t="n">
-        <v>0</v>
+      <c r="C153" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="D153" s="25" t="n">
-        <v>0</v>
+        <v>0.01111111111111111</v>
       </c>
     </row>
     <row r="154">
@@ -7023,10 +7023,10 @@
         </is>
       </c>
       <c r="C157" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D157" s="25" t="n">
-        <v>0.04054054054054054</v>
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="158">
@@ -7036,10 +7036,10 @@
         </is>
       </c>
       <c r="C158" s="6" t="n">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="D158" s="25" t="n">
-        <v>0.9459459459459459</v>
+        <v>0.9333333333333333</v>
       </c>
     </row>
     <row r="159">
@@ -7090,7 +7090,7 @@
         <v>3</v>
       </c>
       <c r="D162" s="25" t="n">
-        <v>0.04054054054054054</v>
+        <v>0.03333333333333333</v>
       </c>
     </row>
     <row r="163">
@@ -7100,10 +7100,10 @@
         </is>
       </c>
       <c r="C163" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D163" s="25" t="n">
-        <v>0.01351351351351351</v>
+        <v>0.02222222222222222</v>
       </c>
     </row>
     <row r="164">
@@ -7154,7 +7154,7 @@
         <v>1</v>
       </c>
       <c r="D167" s="25" t="n">
-        <v>0.01351351351351351</v>
+        <v>0.01111111111111111</v>
       </c>
     </row>
     <row r="168">
@@ -7167,7 +7167,7 @@
         <v>5</v>
       </c>
       <c r="D168" s="25" t="n">
-        <v>0.06756756756756757</v>
+        <v>0.05555555555555555</v>
       </c>
     </row>
     <row r="169">
@@ -7193,7 +7193,7 @@
         <v>3</v>
       </c>
       <c r="D170" s="25" t="n">
-        <v>0.04054054054054054</v>
+        <v>0.03333333333333333</v>
       </c>
     </row>
     <row r="171">
@@ -7216,10 +7216,10 @@
         </is>
       </c>
       <c r="C172" s="6" t="n">
-        <v>61</v>
+        <v>76</v>
       </c>
       <c r="D172" s="25" t="n">
-        <v>0.8243243243243243</v>
+        <v>0.8444444444444444</v>
       </c>
     </row>
     <row r="173">
@@ -7232,7 +7232,7 @@
         <v>3</v>
       </c>
       <c r="D173" s="25" t="n">
-        <v>0.04054054054054054</v>
+        <v>0.03333333333333333</v>
       </c>
     </row>
     <row r="174">
@@ -7280,10 +7280,10 @@
         </is>
       </c>
       <c r="C177" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D177" s="25" t="n">
-        <v>0.01351351351351351</v>
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="178">
@@ -7293,10 +7293,10 @@
         </is>
       </c>
       <c r="C178" s="6" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="D178" s="25" t="n">
-        <v>0.6081081081081081</v>
+        <v>0.6111111111111112</v>
       </c>
     </row>
     <row r="179">
@@ -7306,10 +7306,10 @@
         </is>
       </c>
       <c r="C179" s="6" t="n">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="D179" s="25" t="n">
-        <v>0.5135135135135135</v>
+        <v>0.5111111111111111</v>
       </c>
     </row>
     <row r="180">
@@ -7319,10 +7319,10 @@
         </is>
       </c>
       <c r="C180" s="6" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="D180" s="25" t="n">
-        <v>0.5675675675675675</v>
+        <v>0.5555555555555556</v>
       </c>
     </row>
     <row r="181">
@@ -7332,10 +7332,10 @@
         </is>
       </c>
       <c r="C181" s="6" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D181" s="25" t="n">
-        <v>0.2567567567567567</v>
+        <v>0.2666666666666667</v>
       </c>
     </row>
     <row r="182">
@@ -7345,10 +7345,10 @@
         </is>
       </c>
       <c r="C182" s="6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D182" s="25" t="n">
-        <v>0.1486486486486487</v>
+        <v>0.1444444444444444</v>
       </c>
     </row>
     <row r="183">
@@ -7358,10 +7358,10 @@
         </is>
       </c>
       <c r="C183" s="6" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D183" s="25" t="n">
-        <v>0.4594594594594595</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="184">
@@ -7371,10 +7371,10 @@
         </is>
       </c>
       <c r="C184" s="6" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D184" s="25" t="n">
-        <v>0.1351351351351351</v>
+        <v>0.1222222222222222</v>
       </c>
     </row>
     <row r="185">
@@ -7387,7 +7387,7 @@
         <v>4</v>
       </c>
       <c r="D185" s="25" t="n">
-        <v>0.05405405405405406</v>
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="186">
@@ -7400,7 +7400,7 @@
         <v>5</v>
       </c>
       <c r="D186" s="25" t="n">
-        <v>0.06756756756756757</v>
+        <v>0.05555555555555555</v>
       </c>
     </row>
     <row r="187">
@@ -7448,10 +7448,10 @@
         </is>
       </c>
       <c r="C190" s="6" t="n">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="D190" s="25" t="n">
-        <v>0.7432432432432432</v>
+        <v>0.7666666666666667</v>
       </c>
     </row>
     <row r="191">
@@ -7461,10 +7461,10 @@
         </is>
       </c>
       <c r="C191" s="6" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="D191" s="25" t="n">
-        <v>0.2432432432432433</v>
+        <v>0.2777777777777778</v>
       </c>
     </row>
     <row r="192">
@@ -7474,10 +7474,10 @@
         </is>
       </c>
       <c r="C192" s="6" t="n">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="D192" s="25" t="n">
-        <v>0.2972972972972973</v>
+        <v>0.3555555555555556</v>
       </c>
     </row>
     <row r="193">
@@ -7487,10 +7487,10 @@
         </is>
       </c>
       <c r="C193" s="6" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="D193" s="25" t="n">
-        <v>0.2702702702702703</v>
+        <v>0.3111111111111111</v>
       </c>
     </row>
     <row r="194">
@@ -7500,10 +7500,10 @@
         </is>
       </c>
       <c r="C194" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D194" s="25" t="n">
-        <v>0.04054054054054054</v>
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="195">
@@ -7513,10 +7513,10 @@
         </is>
       </c>
       <c r="C195" s="6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D195" s="25" t="n">
-        <v>0.08108108108108109</v>
+        <v>0.08888888888888889</v>
       </c>
     </row>
     <row r="196">
@@ -7526,10 +7526,10 @@
         </is>
       </c>
       <c r="C196" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D196" s="25" t="n">
-        <v>0.1081081081081081</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="197">
@@ -7539,10 +7539,10 @@
         </is>
       </c>
       <c r="C197" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D197" s="25" t="n">
-        <v>0.1216216216216216</v>
+        <v>0.1333333333333333</v>
       </c>
     </row>
     <row r="198">
@@ -7590,10 +7590,10 @@
         </is>
       </c>
       <c r="C201" s="6" t="n">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="D201" s="25" t="n">
-        <v>0.581081081081081</v>
+        <v>0.5777777777777777</v>
       </c>
     </row>
     <row r="202">
@@ -7603,10 +7603,10 @@
         </is>
       </c>
       <c r="C202" s="6" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D202" s="25" t="n">
-        <v>0.2567567567567567</v>
+        <v>0.2666666666666667</v>
       </c>
     </row>
     <row r="203">
@@ -7616,10 +7616,10 @@
         </is>
       </c>
       <c r="C203" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D203" s="25" t="n">
-        <v>0.1486486486486487</v>
+        <v>0.1333333333333333</v>
       </c>
     </row>
     <row r="204">
@@ -7667,10 +7667,10 @@
         </is>
       </c>
       <c r="C207" s="6" t="n">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="D207" s="25" t="n">
-        <v>0.6351351351351351</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="208">
@@ -7680,10 +7680,10 @@
         </is>
       </c>
       <c r="C208" s="6" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="D208" s="25" t="n">
-        <v>0.3513513513513514</v>
+        <v>0.3777777777777778</v>
       </c>
     </row>
     <row r="209">
@@ -7731,10 +7731,10 @@
         </is>
       </c>
       <c r="C212" s="6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D212" s="25" t="n">
-        <v>0.1081081081081081</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="213">
@@ -7744,10 +7744,10 @@
         </is>
       </c>
       <c r="C213" s="6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D213" s="25" t="n">
-        <v>0.2837837837837838</v>
+        <v>0.2444444444444444</v>
       </c>
     </row>
     <row r="214">
@@ -7757,10 +7757,10 @@
         </is>
       </c>
       <c r="C214" s="6" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D214" s="25" t="n">
-        <v>0.1621621621621622</v>
+        <v>0.1555555555555556</v>
       </c>
     </row>
     <row r="215">
@@ -7770,10 +7770,10 @@
         </is>
       </c>
       <c r="C215" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D215" s="25" t="n">
-        <v>0.05405405405405406</v>
+        <v>0.05555555555555555</v>
       </c>
     </row>
     <row r="216">
@@ -7783,10 +7783,10 @@
         </is>
       </c>
       <c r="C216" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D216" s="25" t="n">
-        <v>0.02702702702702703</v>
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="217">
@@ -7834,10 +7834,10 @@
         </is>
       </c>
       <c r="C220" s="6" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D220" s="25" t="n">
-        <v>0.2567567567567567</v>
+        <v>0.2555555555555555</v>
       </c>
     </row>
     <row r="221">
@@ -7850,7 +7850,7 @@
         <v>1</v>
       </c>
       <c r="D221" s="25" t="n">
-        <v>0.01351351351351351</v>
+        <v>0.01111111111111111</v>
       </c>
     </row>
     <row r="222">
@@ -7863,7 +7863,7 @@
         <v>3</v>
       </c>
       <c r="D222" s="25" t="n">
-        <v>0.04054054054054054</v>
+        <v>0.03333333333333333</v>
       </c>
     </row>
     <row r="223">
@@ -7873,10 +7873,10 @@
         </is>
       </c>
       <c r="C223" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D223" s="25" t="n">
-        <v>0.05405405405405406</v>
+        <v>0.05555555555555555</v>
       </c>
     </row>
     <row r="224">
@@ -7889,7 +7889,7 @@
         <v>3</v>
       </c>
       <c r="D224" s="25" t="n">
-        <v>0.04054054054054054</v>
+        <v>0.03333333333333333</v>
       </c>
     </row>
     <row r="225">
@@ -7899,10 +7899,10 @@
         </is>
       </c>
       <c r="C225" s="6" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="D225" s="25" t="n">
-        <v>0.3918918918918919</v>
+        <v>0.3888888888888889</v>
       </c>
     </row>
     <row r="226">
@@ -7912,10 +7912,10 @@
         </is>
       </c>
       <c r="C226" s="6" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D226" s="25" t="n">
-        <v>0.1891891891891892</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="227">
@@ -7963,10 +7963,10 @@
         </is>
       </c>
       <c r="C230" s="6" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D230" s="25" t="n">
-        <v>0.2837837837837838</v>
+        <v>0.2888888888888889</v>
       </c>
     </row>
     <row r="231">
@@ -7976,10 +7976,10 @@
         </is>
       </c>
       <c r="C231" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D231" s="25" t="n">
-        <v>0.05405405405405406</v>
+        <v>0.05555555555555555</v>
       </c>
     </row>
     <row r="232">
@@ -8005,7 +8005,7 @@
         <v>1</v>
       </c>
       <c r="D233" s="25" t="n">
-        <v>0.01351351351351351</v>
+        <v>0.01111111111111111</v>
       </c>
     </row>
     <row r="234">
@@ -8028,10 +8028,10 @@
         </is>
       </c>
       <c r="C235" s="6" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="D235" s="25" t="n">
-        <v>0.7432432432432432</v>
+        <v>0.7222222222222222</v>
       </c>
     </row>
     <row r="236">
@@ -8079,10 +8079,10 @@
         </is>
       </c>
       <c r="C239" s="6" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D239" s="25" t="n">
-        <v>0.1486486486486487</v>
+        <v>0.1777777777777778</v>
       </c>
     </row>
     <row r="240">
@@ -8092,10 +8092,10 @@
         </is>
       </c>
       <c r="C240" s="6" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D240" s="25" t="n">
-        <v>0.1621621621621622</v>
+        <v>0.1777777777777778</v>
       </c>
     </row>
     <row r="241">
@@ -8108,7 +8108,7 @@
         <v>4</v>
       </c>
       <c r="D241" s="25" t="n">
-        <v>0.05405405405405406</v>
+        <v>0.04444444444444445</v>
       </c>
     </row>
     <row r="242">
@@ -8121,7 +8121,7 @@
         <v>5</v>
       </c>
       <c r="D242" s="25" t="n">
-        <v>0.06756756756756757</v>
+        <v>0.05555555555555555</v>
       </c>
     </row>
     <row r="243">
@@ -8178,7 +8178,7 @@
       </c>
       <c r="C247" s="32" t="inlineStr">
         <is>
-          <t>4.0 Years</t>
+          <t>4.1 Years</t>
         </is>
       </c>
     </row>
@@ -8190,7 +8190,7 @@
       </c>
       <c r="C248" s="32" t="inlineStr">
         <is>
-          <t>3.2 Years</t>
+          <t>3.4 Years</t>
         </is>
       </c>
     </row>
@@ -8202,7 +8202,7 @@
       </c>
       <c r="C249" s="32" t="inlineStr">
         <is>
-          <t>4.7 Years</t>
+          <t>4.9 Years</t>
         </is>
       </c>
     </row>

</xml_diff>